<commit_message>
Layout Rev Done - NO DRC Check
</commit_message>
<xml_diff>
--- a/hw/PIB/monarch_payload_interface_board_rev2/PIB STM32 Pinouts.xlsx
+++ b/hw/PIB/monarch_payload_interface_board_rev2/PIB STM32 Pinouts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\monarch-payload-interface-board\hw\PIB\monarch_payload_interface_board_rev2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FB39C2-D9D9-4ACB-B0B4-7D1965F89B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677CF8A4-FEDD-460D-84DB-072ABCD17652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{362559DF-8766-43DC-9949-A5C2C567812D}"/>
+    <workbookView xWindow="5772" yWindow="372" windowWidth="11712" windowHeight="13776" xr2:uid="{362559DF-8766-43DC-9949-A5C2C567812D}"/>
   </bookViews>
   <sheets>
     <sheet name="Pinout Descriptions" sheetId="1" r:id="rId1"/>

</xml_diff>